<commit_message>
Add new patient fields
</commit_message>
<xml_diff>
--- a/docs/samples/patient_upload_template.xlsx
+++ b/docs/samples/patient_upload_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,6 +442,141 @@
           <t>Gender</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Street Address</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Zip</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Emergency Contact Name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Emergency Contact Relationship</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Emergency Contact Phone</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Preferred Language</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Race/Ethnicity</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Marital Status</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Occupation</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Insurance Provider</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Policy Number</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>PCP Name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Registration Date</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Preferred Pharmacy</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Blood Type</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Height (in)</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Weight (lbs)</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Allergies</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Current Medications</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Chronic Conditions (ICD-10)</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Immunization History</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Smoking Status</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Alcohol Use</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -469,6 +604,33 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add patient analytics dashboard (data overview + visualizations)
</commit_message>
<xml_diff>
--- a/docs/samples/patient_upload_template.xlsx
+++ b/docs/samples/patient_upload_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AJ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,55 +524,75 @@
       </c>
       <c r="V1" t="inlineStr">
         <is>
+          <t>Care Department</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>Registration Date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Last Visit Date</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Preferred Pharmacy</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Blood Type</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Height (in)</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Weight (lbs)</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Systolic BP</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Diastolic BP</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Allergies</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Current Medications</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Chronic Conditions (ICD-10)</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Immunization History</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Smoking Status</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Alcohol Use</t>
         </is>
@@ -631,6 +651,10 @@
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>